<commit_message>
adding deme 2 results
</commit_message>
<xml_diff>
--- a/DDM GD Find Alpha Rebuild/all_deme_alpha_results_summary.xlsx
+++ b/DDM GD Find Alpha Rebuild/all_deme_alpha_results_summary.xlsx
@@ -8,19 +8,30 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Moar Documents\GitHub\Bac_Evol_SSA\DDM GD Find Alpha Rebuild\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{829FB338-B0F7-4429-9B64-84D5B3EBF17A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B523454-9FFD-469F-80B8-C3FE5102C577}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
     <t>deme_index</t>
   </si>
@@ -62,6 +73,9 @@
   </si>
   <si>
     <t>stderr_ci_final</t>
+  </si>
+  <si>
+    <t>alpha_star * slope_final</t>
   </si>
 </sst>
 </file>
@@ -425,7 +439,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N102"/>
+  <dimension ref="A1:O102"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.140625" bestFit="1" customWidth="1"/>
@@ -437,9 +451,10 @@
     <col min="12" max="12" width="12.85546875" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="12.28515625" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="14" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="22.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -482,8 +497,11 @@
       <c r="N1" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O1" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -526,13 +544,60 @@
       <c r="N2">
         <v>20000</v>
       </c>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O2">
+        <f>F2*C2</f>
+        <v>0.20448449049130338</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="B3">
+        <v>8.7437268462869769E-2</v>
+      </c>
+      <c r="C3">
+        <v>14453.8359375</v>
+      </c>
+      <c r="D3">
+        <v>8.5707925260066986E-2</v>
+      </c>
+      <c r="E3">
+        <v>1.5211037862172819E-5</v>
+      </c>
+      <c r="F3">
+        <v>8.6147456386242993E-6</v>
+      </c>
+      <c r="G3">
+        <v>11250</v>
+      </c>
+      <c r="H3">
+        <v>15750</v>
+      </c>
+      <c r="I3">
+        <v>0.55271226167678833</v>
+      </c>
+      <c r="J3">
+        <v>0.30549082159996033</v>
+      </c>
+      <c r="K3">
+        <v>7.8165316954255104E-3</v>
+      </c>
+      <c r="L3">
+        <v>19679.36422429252</v>
+      </c>
+      <c r="M3">
+        <v>300</v>
+      </c>
+      <c r="N3">
+        <v>20000</v>
+      </c>
+      <c r="O3">
+        <f t="shared" ref="O3:O4" si="0">F3*C3</f>
+        <v>0.12451612010396929</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -575,63 +640,67 @@
       <c r="N4">
         <v>20000</v>
       </c>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O4">
+        <f t="shared" si="0"/>
+        <v>0.16031380495593517</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>15</v>
       </c>

</xml_diff>